<commit_message>
Anchor: LibreOffice upstream/master@2026-09-16 (534ed0054465b3bb0742c148876164ac14e598b3)
</commit_message>
<xml_diff>
--- a/sc/qa/unit/data/xlsx/twoCellAnchor_editAs_oneCell.xlsx
+++ b/sc/qa/unit/data/xlsx/twoCellAnchor_editAs_oneCell.xlsx
@@ -2,17 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\bugtesting\OTRS\1006330\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
+  <workbookPr filterPrivacy="1" defaultThemeVersion="153222"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16275" windowHeight="7275"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="16272" windowHeight="7272"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
+    <sheet name="Tabelle2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="152511" iterateDelta="1E-4"/>
   <extLst>
@@ -59,7 +55,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -112,6 +108,55 @@
         <a:xfrm>
           <a:off x="0" y="2"/>
           <a:ext cx="4352924" cy="2743198"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>716118</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>54163</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>182716</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>150366</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Grafik 1"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm rot="14400000">
+          <a:off x="248915" y="887126"/>
+          <a:ext cx="3570923" cy="2636518"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -387,9 +432,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>